<commit_message>
Enables overpayment to credit functionality
Implements the functionality to transfer overpaid amounts from a payment to the customer's credit.

This change includes:

- An endpoint to handle the transfer of overpaid funds.
- Validation to ensure the payment is actually overpaid before transferring funds.
- Creation of an internal transaction to record the transfer.
- Role-based authorization to allow only accountants and admins to perform this action.
- Updates payment status to 'Paid' after overpayment is credited

Fixes #71
</commit_message>
<xml_diff>
--- a/ErrorCodes.xlsx
+++ b/ErrorCodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zamos\Documents\GitHub\CtrlPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E95975F-B2E0-45DB-B70D-8C0CF00E47ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3414CF-CDDA-4CED-9AA5-AEB340ABBDBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38115" yWindow="5595" windowWidth="28800" windowHeight="15345" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38115" yWindow="5595" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Auth" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="111">
   <si>
     <t>user with the same username already exists</t>
   </si>
@@ -359,6 +359,9 @@
   </si>
   <si>
     <t>operation successful</t>
+  </si>
+  <si>
+    <t>payment is not overpaid</t>
   </si>
 </sst>
 </file>
@@ -1059,13 +1062,13 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="WARNING">
+    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="WARNING">
       <formula>NOT(ISERROR(SEARCH("WARNING",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="ERROR">
+    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1153,6 +1156,12 @@
       <c r="A7" t="s">
         <v>76</v>
       </c>
+      <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1207,13 +1216,13 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="WARNING">
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="WARNING">
       <formula>NOT(ISERROR(SEARCH("WARNING",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="ERROR">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1361,13 +1370,13 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="WARNING">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="WARNING">
       <formula>NOT(ISERROR(SEARCH("WARNING",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="ERROR">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1491,13 +1500,13 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="OK">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="WARNING">
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="WARNING">
       <formula>NOT(ISERROR(SEARCH("WARNING",C1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="ERROR">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="ERROR">
       <formula>NOT(ISERROR(SEARCH("ERROR",C1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Introduces admin and loyal customer management
Adds an admin API for listing users and a transaction API for viewing all transactions, both secured with role-based authorization.

Enhances the loyal customer promotion process by generating unique registration codes and sending automated email notifications using new Razor-based mail templates and a dedicated mail rendering service.

Updates the user registration flow to require a valid loyal customer code, linking new user accounts to their respective loyal customer profiles.

Refactors repository names from `AccountantPaymentRepo` to `AccountantRepo` and `ToDoRepo` to `AdminRepo` for better clarity and organization, updating frontend components to reflect these changes.

Introduces new DTOs for user data and refines existing customer DTOs to support the new functionalities.
</commit_message>
<xml_diff>
--- a/ErrorCodes.xlsx
+++ b/ErrorCodes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zamos\Documents\GitHub\CtrlPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3414CF-CDDA-4CED-9AA5-AEB340ABBDBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B757EE-754E-42B3-B56D-E827D6380A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38115" yWindow="5595" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13065" yWindow="5475" windowWidth="28800" windowHeight="15345" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Auth" sheetId="2" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="112">
   <si>
     <t>user with the same username already exists</t>
   </si>
@@ -362,6 +362,9 @@
   </si>
   <si>
     <t>payment is not overpaid</t>
+  </si>
+  <si>
+    <t>code is not valid</t>
   </si>
 </sst>
 </file>
@@ -1321,6 +1324,12 @@
       <c r="A8" t="s">
         <v>39</v>
       </c>
+      <c r="B8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">

</xml_diff>